<commit_message>
Update milk exports (auto)
</commit_message>
<xml_diff>
--- a/data/prozorro-milk.xlsx
+++ b/data/prozorro-milk.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-01-09T14:13:30+00:00</t>
+          <t>2026-01-10T04:04:15+00:00</t>
         </is>
       </c>
     </row>
@@ -500,13 +500,13 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>{
-  "offset": "1478282081.222461.1.aa27d5a4cff39529aed6b77e05a4f515",
-  "updated_at": "2026-01-09T14:13:30.494741+00:00",
-  "pages_done": 100,
-  "tenders_scanned": 10000,
-  "tenders_fetched": 10000,
-  "milk_tenders": 101,
-  "milk_items": 105
+  "offset": "1478282201.539197.1.a66672a13d1cb6ac87a6aa2598195569",
+  "updated_at": "2026-01-10T04:04:14.647870+00:00",
+  "pages_done": 125,
+  "tenders_scanned": 12500,
+  "tenders_fetched": 12500,
+  "milk_tenders": 105,
+  "milk_items": 109
 }</t>
         </is>
       </c>
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M106"/>
+  <dimension ref="A1:M110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7323,6 +7323,218 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>bf560e6205534e159a359e2f44638f6e</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>7c1701269f544ed18f34fbbe83962e7e</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>10.51.1 Молоко та вершки, рідинні, оброблені (10.51.11-42.00 молоко)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>15510000-6</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>2</v>
+      </c>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:55:07.272506+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>e8354bf0d23b4ff58d9492de3d537b95</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>e5433dcde8634970a4e277c9342e3100</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Молоко та вершки рідинні, оброблені</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>15512000-0</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>штуки</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>2015-12-31T23:59:59.999999+02:00</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>м. Київ</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:55:29.388767+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>3ad3c0ec445a459f905c9e566cccfdda</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>9ac2fc11687f4b1ea971ff04d5906b12</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Молоко питне ультрапастеризоване за кодом ДК 016:2010 – 10.51.1- «Молоко та вершки, рідинні, оброблені»</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>15511100-4</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>4495</v>
+      </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:55:37.273894+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>9373b16c10bc4c89b1a584fba7054422</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>bdf926b898d7446fa918f262fc1f2e16</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>1.	Кава у зернах, 500 гр	30 	шт 2.	Цукор пресований у кубиках (500 г)	10 	шт 3.	 Вершки сухі для напоїв Coffee-mate, 400 гр.	10 	шт 4.	Серветки столові білі, одношарові, в упаковці 500 штук	10 	шт 5.	 Чай зелений Greenfield Flying Dragon, в упаковці 100 пак.	5 	шт 6.	 Чай чорний Greenfield Golden Ceylon, в упаковці 100 пак.	5 	шт 7.	Цукор-пісок, 1 кг	10 	шт 8.	Палички для розмішування напоїв, в упаковці 1000 шт.	5  	шт</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>15860000-4</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>85</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>штуки</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2015-08-10T00:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>2015-08-11T23:59:59.999999+03:00</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Київськая</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>м. Київ</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:56:11.256963+02:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7334,7 +7546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K102"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12744,6 +12956,218 @@
       <c r="K102" t="inlineStr">
         <is>
           <t>2026-01-09T14:12:54.405696+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>bf560e6205534e159a359e2f44638f6e</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>UA-2015-07-07-000020</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:55:07.272506+02:00</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>unsuccessful</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Відокремлений підрозділ "Донбаська електроенергетична система" ДП "НЕК "Укренерго"</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>23344104</t>
+        </is>
+      </c>
+      <c r="H103" t="n">
+        <v>20160</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>1</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:03:23.262021+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>e8354bf0d23b4ff58d9492de3d537b95</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>UA-2015-07-14-000086</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:55:29.388767+02:00</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>ДП "Київська міська дирекція УДППЗ "Укрпошта""</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>01189979</t>
+        </is>
+      </c>
+      <c r="H104" t="n">
+        <v>12000</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>1</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:03:23.262021+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>3ad3c0ec445a459f905c9e566cccfdda</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>UA-2015-07-17-000044</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:55:37.273894+02:00</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Білгород-Дністровська філія державного підпириємства "Адміністрація морських портів України" (адміністрація Білгород-Дністровського морського порту)</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>38728376</t>
+        </is>
+      </c>
+      <c r="H105" t="n">
+        <v>24497.75</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>0</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:03:23.262021+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>9373b16c10bc4c89b1a584fba7054422</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>UA-2015-07-28-000156</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:56:11.256963+02:00</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>active.awarded</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>ДП "УКРІНТЕРАВТОСЕРВІС"</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>21536845</t>
+        </is>
+      </c>
+      <c r="H106" t="n">
+        <v>4340</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>1</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:03:23.262021+00:00</t>
         </is>
       </c>
     </row>
@@ -12758,7 +13182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12919,6 +13343,164 @@
       </c>
       <c r="E6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-01-09T14:13:30+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>XLSX export done</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{"bytes": 39861}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:04:15+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Start XLSX export</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"db": "data/prozorro_milk.sqlite", "xlsx": "data/prozorro-milk.xlsx"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:04:15+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Discovered tables</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{"tables": ["milk_items", "milk_tenders"]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:04:15+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Export table</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{"table": "milk_items"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:04:15+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Export table</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{"table": "milk_tenders"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:04:15+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Attach logs sheet</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update XLSX with logs (auto)
</commit_message>
<xml_diff>
--- a/data/prozorro-milk.xlsx
+++ b/data/prozorro-milk.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-01-10T04:04:15+00:00</t>
+          <t>2026-01-11T04:18:58+00:00</t>
         </is>
       </c>
     </row>
@@ -500,13 +500,13 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>{
-  "offset": "1478282201.539197.1.a66672a13d1cb6ac87a6aa2598195569",
-  "updated_at": "2026-01-10T04:04:14.647870+00:00",
-  "pages_done": 125,
-  "tenders_scanned": 12500,
-  "tenders_fetched": 12500,
-  "milk_tenders": 105,
-  "milk_items": 109
+  "offset": "1478282349.043586.1.d0a1099efcee93f25a6d54a870cbb3fb",
+  "updated_at": "2026-01-11T04:18:58.154506+00:00",
+  "pages_done": 150,
+  "tenders_scanned": 15000,
+  "tenders_fetched": 15000,
+  "milk_tenders": 122,
+  "milk_items": 126
 }</t>
         </is>
       </c>
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M110"/>
+  <dimension ref="A1:M127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7535,6 +7535,883 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>916a88cc63914fccb0b4f64c30c21448</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>94a4eff26f8d41e2ac8176da6a026476</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>молоко коров’яче питне пастеризоване жирністю 2,5% (код 10.51.1 згідно ДК 016-2010 Молоко та вершки рідинні, оброблені)</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>15511100-4</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>10300</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>кілограми</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>KGM</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2015-09-30T21:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>2015-12-27T22:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Хмельницька</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:56:54.645091+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ca282f2cafb64b7eb7bfd9c7444729e9</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>d6b5655ca6c3436e9ed14ef3a5100c9b</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>«Молоко та вершки, рідинні, оброблені» (молоко).</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>15511000-3</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>літр</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>LTR</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>2015-09-20T21:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>2015-12-30T22:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Запорізька</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:56:56.948559+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>0501d112b17740179b6dfe222d741b2f</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>d8276df064874ad99ad611a109b11e40</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Молоко фас 1 літр п/е, 2.5%</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>15511100-4</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>8700</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>штуки</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2015-08-24T00:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>2015-12-31T23:59:59.999999+02:00</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:56:59.231733+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>9cc032b602cc46e6b2d6d2837ea41dba</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>f366ed4468884fe3913bf24ab5e82124</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Молоко та вершки, рідинні, оброблені</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>15510000-6</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>LTR</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ДНЕПРОПЕТРОВСКАЯ ОБЛ.</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Днепропетровск</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:06.394159+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>9407598a5564447381e1ee10856e3668</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>6fa3b4421be64b31be89a1707220e910</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Молоко 2,5 % поліетилен 1 л</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>15510000-6</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>600</v>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:14.626309+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>b4e8d08a57e848238c6cc2cca30bf223</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>ad13743cfee3465fbbb6abde5a77ef53</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Молоко 2,5 % поліетилен 1 л</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>15511000-3</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>600</v>
+      </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:14.814561+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>0161f1d8ae954179af635e147f4cbf74</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>606b65025a6f466c87d663620629c54e</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Молоко 3,2 % пастеризоване поліетилен 0,5 л</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>15511100-4</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>600</v>
+      </c>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:33.478429+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>dff9746856564cd2b249d8612a56fa43</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>17748e8984184102b9e14950a033c317</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Молоко 2,5 % пастеризоване поліетилен  1 л</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>15511100-4</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>450</v>
+      </c>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:33.624524+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>eeea13766d6b49c2b30087060f6573e3</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>12af1eef216343a4ad29a76a14122b4d</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Молоко 2,5 % поліетилен  0,5 л</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>15511000-3</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>2082</v>
+      </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:34.294837+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>89c1f871adc44165a78dec1a036dc3db</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>5971f193a4214591b2bd526f1465b812</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Молоко 2,5 % поліетилен  0,5 л</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>15511000-3</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>3920</v>
+      </c>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:37.074563+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>20fc3534a32e4e98a37e1fc41ce4adb8</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>4b49b8426886471a89bcf13d76ec9d9b</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Молоко пастеризоване 2.7% 500г.</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>15511100-4</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>1102</v>
+      </c>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:42.706161+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>c9a4c99b475342b1b3e707cafd1feea3</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>c3cef331746e42af9d3dc2024028f064</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>молоко 2,5 % жир.(10.51.11-42.00)</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>15510000-6</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>22360</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>литр</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>LTR</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:58:04.492396+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>fca11035a4d742b1b9efb53c84254420</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>d70a355ef0c048b4b14b06b3a69894c6</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Молоко пастеризоване 2,5%</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>03000000-1</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>литр</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>LTR</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Київська</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:58:21.863187+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>05b4cac24a3d43bf95917a444541ba85</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>6b50aa94de2045a09f7f008672b70b78</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>молоко сухе знежирене</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>15511000-3</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>500</v>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>кілограми</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>KGM</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2015-11-01T22:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>2015-11-29T22:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Рівненська</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:58:34.794793+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>8aea2333476c49ef8249f9cf7208fc80</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>be7fb4b2a8e347399d423d1926f86cf2</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Молоко 2,6 % жирность ДСТУ 2661-94</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>42000000-6</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>32000</v>
+      </c>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ХАРЬКОВСКАЯ ОБЛ.</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Харьков</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:58:39.134971+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>fb24e47fbd424063be7640428411abca</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>a214e419e3b74caf95a6393467937c83</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Молоко тривалого зберігання 2,6% 1 л</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>15511100-4</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>65</v>
+      </c>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>H87</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:59:08.100157+02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>a87b459aa61d4bb0876a8f142170b2bb</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>6d90ce275da046bca5a0e9412e15dea3</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>молоко жирність 2,6% плівка по 1л</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>15510000-6</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>4450</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>літр</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>LTR</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2015-09-24T21:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>2015-12-30T22:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Київська</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:59:08.363048+02:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7546,7 +8423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K106"/>
+  <dimension ref="A1:K123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13168,6 +14045,907 @@
       <c r="K106" t="inlineStr">
         <is>
           <t>2026-01-10T04:03:23.262021+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>916a88cc63914fccb0b4f64c30c21448</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>UA-2015-08-10-000028</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:56:54.645091+02:00</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>unsuccessful</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>ВП ХАЕС ДП "НАЕК "Енергоатом"</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>21313677</t>
+        </is>
+      </c>
+      <c r="H107" t="n">
+        <v>92700</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>1</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>ca282f2cafb64b7eb7bfd9c7444729e9</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>UA-2015-08-11-000019</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:56:56.948559+02:00</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>ВП Запорізька АЕС ДП НАЕК "Енергоатом"</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>19355964</t>
+        </is>
+      </c>
+      <c r="H108" t="n">
+        <v>31486</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>1</v>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>0501d112b17740179b6dfe222d741b2f</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>UA-2015-08-11-000073</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:56:59.231733+02:00</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Київська міська дитяча клінічна лікарня № 2</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>05415941</t>
+        </is>
+      </c>
+      <c r="H109" t="n">
+        <v>99750</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>1</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>9cc032b602cc46e6b2d6d2837ea41dba</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>UA-2015-08-12-000118</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:06.394159+02:00</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>unsuccessful</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Придніпровська залізниця"</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>01073828</t>
+        </is>
+      </c>
+      <c r="H110" t="n">
+        <v>20500</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>1</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>9407598a5564447381e1ee10856e3668</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>UA-2015-08-14-000057</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:14.626309+02:00</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>unsuccessful</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Придніпровська залізниця"</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>01073828</t>
+        </is>
+      </c>
+      <c r="H111" t="n">
+        <v>5700</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>1</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>b4e8d08a57e848238c6cc2cca30bf223</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>UA-2015-08-14-000061</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:14.814561+02:00</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Придніпровська залізниця"</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>01073828</t>
+        </is>
+      </c>
+      <c r="H112" t="n">
+        <v>5700</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>1</v>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>0161f1d8ae954179af635e147f4cbf74</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>UA-2015-08-19-000071</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:33.478429+02:00</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Придніпровська залізниця"</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>01073828</t>
+        </is>
+      </c>
+      <c r="H113" t="n">
+        <v>3360</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>1</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>dff9746856564cd2b249d8612a56fa43</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>UA-2015-08-19-000078</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:33.624524+02:00</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Придніпровська залізниця"</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>01073828</t>
+        </is>
+      </c>
+      <c r="H114" t="n">
+        <v>8280</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>1</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>eeea13766d6b49c2b30087060f6573e3</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>UA-2015-08-19-000102</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:34.294837+02:00</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>unsuccessful</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Придніпровська залізниця"</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>01073828</t>
+        </is>
+      </c>
+      <c r="H115" t="n">
+        <v>9993.6</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>1</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>89c1f871adc44165a78dec1a036dc3db</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>UA-2015-08-20-000066</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:37.074563+02:00</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Придніпровська залізниця"</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>01073828</t>
+        </is>
+      </c>
+      <c r="H116" t="n">
+        <v>19992</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J116" t="n">
+        <v>1</v>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>20fc3534a32e4e98a37e1fc41ce4adb8</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>UA-2015-08-21-000105</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:57:42.706161+02:00</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>unsuccessful</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Придніпровська залізниця"</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>01073828</t>
+        </is>
+      </c>
+      <c r="H117" t="n">
+        <v>6820</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
+        <v>1</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>c9a4c99b475342b1b3e707cafd1feea3</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>UA-2015-08-28-000048</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:58:04.492396+02:00</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Київський національний університет імені Тараса Шевченка</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>02070944</t>
+        </is>
+      </c>
+      <c r="H118" t="n">
+        <v>178880</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J118" t="n">
+        <v>1</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>fca11035a4d742b1b9efb53c84254420</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>UA-2015-09-01-000137</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:58:21.863187+02:00</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>КМКЛ № 4</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>30212155</t>
+        </is>
+      </c>
+      <c r="H119" t="n">
+        <v>28800</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J119" t="n">
+        <v>1</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>05b4cac24a3d43bf95917a444541ba85</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>UA-2015-09-03-000113</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:58:34.794793+02:00</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>unsuccessful</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>відокремлений підрозділ „Рівненська АЕС” державного підприємства   „Національна атомна енергогенеруюча компанія “Енергоатом”</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>05425046</t>
+        </is>
+      </c>
+      <c r="H120" t="n">
+        <v>33000</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J120" t="n">
+        <v>1</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>8aea2333476c49ef8249f9cf7208fc80</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>UA-2015-09-04-000028</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:58:39.134971+02:00</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Український державний центр по експлуатації спеціалізованих вагонів"</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>01056362</t>
+        </is>
+      </c>
+      <c r="H121" t="n">
+        <v>368000</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J121" t="n">
+        <v>1</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>fb24e47fbd424063be7640428411abca</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>UA-2015-09-08-000196</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:59:08.100157+02:00</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>active.awarded</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Державне підприємство "Придніпровська залізниця"</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>01073828</t>
+        </is>
+      </c>
+      <c r="H122" t="n">
+        <v>806</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J122" t="n">
+        <v>1</v>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>a87b459aa61d4bb0876a8f142170b2bb</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>UA-2015-09-08-000199</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>2016-11-04T19:59:08.363048+02:00</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>belowThreshold</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Київська міська клінічна лікарня №8</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>05497146</t>
+        </is>
+      </c>
+      <c r="H123" t="n">
+        <v>46800</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>UAH</t>
+        </is>
+      </c>
+      <c r="J123" t="n">
+        <v>0</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:19.183418+00:00</t>
         </is>
       </c>
     </row>
@@ -13182,7 +14960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13501,6 +15279,164 @@
       </c>
       <c r="E12" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-01-10T04:04:15+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>XLSX export done</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{"bytes": 41407}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:58+00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Start XLSX export</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{"db": "data/prozorro_milk.sqlite", "xlsx": "data/prozorro-milk.xlsx"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:58+00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Discovered tables</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{"tables": ["milk_items", "milk_tenders"]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:58+00:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Export table</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{"table": "milk_items"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:58+00:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Export table</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{"table": "milk_tenders"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-01-11T04:18:58+00:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>normalize</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Attach logs sheet</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>